<commit_message>
Fix example Excel formula display to SOMA(B6:BU6)
Co-authored-by: cafla19791-tech <cafla19791-tech@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/rtn/aba_1_2A_totais_por_item.xlsx
+++ b/output/rtn/aba_1_2A_totais_por_item.xlsx
@@ -4913,7 +4913,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>SOMA(B:BU6)</t>
+          <t>SOMA(B6:BU6)</t>
         </is>
       </c>
     </row>
@@ -4943,7 +4943,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>SOMA(BV:HZ6)</t>
+          <t>SOMA(BV6:HZ6)</t>
         </is>
       </c>
     </row>
@@ -4973,7 +4973,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>SOMA(IA:JE6)</t>
+          <t>SOMA(IA6:JE6)</t>
         </is>
       </c>
     </row>
@@ -5003,7 +5003,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>SOMA(JF:LA6)</t>
+          <t>SOMA(JF6:LA6)</t>
         </is>
       </c>
     </row>
@@ -5033,7 +5033,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>SOMA(LB:MP6)</t>
+          <t>SOMA(LB6:MP6)</t>
         </is>
       </c>
     </row>

</xml_diff>